<commit_message>
se pone el correo de final de entrega
</commit_message>
<xml_diff>
--- a/pruebaDatos.xlsx
+++ b/pruebaDatos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mercadotecnia/Desktop/automatizacióncorreos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E34C272-E796-EE42-A840-D6C21B61E3AB}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A92D51-24C5-714A-8763-CA3511EA2402}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2600" yWindow="3300" windowWidth="27640" windowHeight="16940" xr2:uid="{66D09105-B21B-F042-BD54-AE668A6F427D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>FOLIO DE KIT</t>
   </si>
@@ -52,18 +52,6 @@
   </si>
   <si>
     <t>Central de Autobuses del Norte</t>
-  </si>
-  <si>
-    <t>FA00003</t>
-  </si>
-  <si>
-    <t>FA00004</t>
-  </si>
-  <si>
-    <t>FA00005</t>
-  </si>
-  <si>
-    <t>FA00006</t>
   </si>
 </sst>
 </file>
@@ -488,51 +476,27 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>